<commit_message>
Enhance Gantt skill: story point summation, blank feature workstreams, auto-fit columns
- Features now display sum of all children's story points
- Feature rows have blank workstream (they span multiple workstreams via children)
- Columns auto-fit based on content length with intelligent min/max bounds
- Regenerated gantt-chart.xlsx with improvements applied

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GAP-AI-FOUNDATION/projects/mediquant/gantt/gantt-chart.xlsx
+++ b/GAP-AI-FOUNDATION/projects/mediquant/gantt/gantt-chart.xlsx
@@ -465,28 +465,28 @@
   <dimension ref="A1:V60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="32" customWidth="1" min="22" max="22"/>
+    <col width="9.6" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
+    <col width="19.2" customWidth="1" min="4" max="4"/>
+    <col width="19.2" customWidth="1" min="5" max="5"/>
+    <col width="9.6" customWidth="1" min="6" max="6"/>
+    <col width="34.8" customWidth="1" min="7" max="7"/>
+    <col width="34.8" customWidth="1" min="8" max="8"/>
+    <col width="34.8" customWidth="1" min="9" max="9"/>
+    <col width="34.8" customWidth="1" min="10" max="10"/>
+    <col width="34.8" customWidth="1" min="11" max="11"/>
+    <col width="34.8" customWidth="1" min="12" max="12"/>
+    <col width="34.8" customWidth="1" min="13" max="13"/>
+    <col width="34.8" customWidth="1" min="14" max="14"/>
+    <col width="34.8" customWidth="1" min="15" max="15"/>
+    <col width="34.8" customWidth="1" min="16" max="16"/>
+    <col width="34.8" customWidth="1" min="17" max="17"/>
+    <col width="34.8" customWidth="1" min="18" max="18"/>
+    <col width="34.8" customWidth="1" min="19" max="19"/>
+    <col width="34.8" customWidth="1" min="20" max="20"/>
+    <col width="34.8" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -637,11 +637,7 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="3" t="n">
         <v>0</v>
       </c>
@@ -682,11 +678,7 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="n">
         <v>0</v>
       </c>
@@ -762,13 +754,9 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
@@ -848,7 +836,7 @@
         </is>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
@@ -883,7 +871,7 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
@@ -918,7 +906,7 @@
         </is>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -988,7 +976,7 @@
         </is>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1023,7 +1011,7 @@
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
@@ -1052,13 +1040,9 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="5" t="n"/>
@@ -1167,13 +1151,9 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="n"/>
@@ -1282,13 +1262,9 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G19" s="5" t="n"/>
       <c r="H19" s="5" t="n"/>
@@ -1572,13 +1548,9 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G27" s="5" t="n"/>
       <c r="H27" s="5" t="n"/>
@@ -1722,11 +1694,7 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3" t="n">
         <v>0</v>
       </c>
@@ -1767,13 +1735,9 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E32" s="3" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G32" s="5" t="n"/>
       <c r="H32" s="5" t="n"/>
@@ -1847,13 +1811,9 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E34" s="3" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="G34" s="5" t="n"/>
       <c r="H34" s="5" t="n"/>
@@ -2067,13 +2027,9 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E40" s="3" t="inlineStr"/>
       <c r="F40" s="3" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G40" s="5" t="n"/>
       <c r="H40" s="5" t="n"/>
@@ -2357,13 +2313,9 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E48" s="3" t="inlineStr"/>
       <c r="F48" s="3" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G48" s="5" t="n"/>
       <c r="H48" s="5" t="n"/>
@@ -2612,13 +2564,9 @@
           <t>Bonnie Bordelon</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
+      <c r="E55" s="3" t="inlineStr"/>
       <c r="F55" s="3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G55" s="5" t="n"/>
       <c r="H55" s="5" t="n"/>

</xml_diff>